<commit_message>
Complete verified Stage 3 local release candidate
</commit_message>
<xml_diff>
--- a/excel/youth-unemployment.xlsx
+++ b/excel/youth-unemployment.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates" sheetId="1" r:id="Rf208c988174c4471"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change 2023-2025" sheetId="2" r:id="R9be36c3bd9604236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R99efa57f74e840ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates" sheetId="1" r:id="Ref9c426481774b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Change 2023-2025" sheetId="2" r:id="R1af30ff953c74bdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="3" r:id="R909a3340ad0b4a77"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3248,7 +3248,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra291d3f24162456d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd7287c70545a439b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4235,7 +4235,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra450e165c9744321"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R78b424b8d5c64b93"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4271,7 +4271,7 @@
         <x:v>Ready</x:v>
       </x:c>
       <x:c r="C2" s="9" t="str">
-        <x:v>The selected youth unemployment rates and reported 2023-2025 changes are directly supported by the corrected ILO report.</x:v>
+        <x:v>Fixed historical scope verified under EL-YU-2026-v1.0.0, reviewed 1 October 2026. This edition is not the latest ILOSTAT vintage.</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
@@ -4307,7 +4307,7 @@
         <x:v>Total youth unemployment rates. Youth refers to ages 15-24. ILO modelled estimates, November 2025.</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6" ht="24" hidden="0" customHeight="1">
       <x:c r="A6" s="9" t="str">
         <x:v>Change source</x:v>
       </x:c>
@@ -4315,7 +4315,7 @@
         <x:v>Figure 1.3</x:v>
       </x:c>
       <x:c r="C6" s="9" t="str">
-        <x:v>Reported percentage-point change by subregion and sex, 2023-2025.</x:v>
+        <x:v>ILO-reported percentage-point changes, 2023-2025. A printed zero is rounded, not proof of exact stability.</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
@@ -4359,7 +4359,7 @@
         <x:v>Use 'worsened or failed to improve in 8 of 11 subregions'</x:v>
       </x:c>
       <x:c r="C10" s="9" t="str">
-        <x:v>Figure 1.3 shows six increases, two unchanged subregions and three decreases. This wording is supported by the detailed evidence.</x:v>
+        <x:v>Figure 1.3 prints six increases, two rounded zeros and three decreases. The 8-of-11 classification excludes World and does not establish statistical significance.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="24" hidden="0" customHeight="1">
@@ -4370,7 +4370,7 @@
         <x:v>Youth unemployment recovery stalled across most subregions between 2023 and 2025</x:v>
       </x:c>
       <x:c r="C11" s="9" t="str">
-        <x:v>Six subregions increased and two recorded no change.</x:v>
+        <x:v>Six subregions have positive reported changes and two have rounded zeros. Unrounded movements and causes remain unknown.</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
@@ -4395,7 +4395,7 @@
         <x:v>Low rates can coexist with inactivity, informality or insecure work.</x:v>
       </x:c>
     </x:row>
-    <x:row r="14" ht="15" hidden="0" customHeight="1">
+    <x:row r="14" ht="24" hidden="0" customHeight="1">
       <x:c r="A14" s="9" t="str">
         <x:v>Global count</x:v>
       </x:c>
@@ -4403,13 +4403,13 @@
         <x:v>Approximately 67 million unemployed youth in 2025</x:v>
       </x:c>
       <x:c r="C14" s="9" t="str">
-        <x:v>Rounded figure from the ILO report and news release; regional counts are not included here.</x:v>
+        <x:v>Approximate rounded headline from section 1.1, printed page 1. Stored as 67,000,000, not an exact individual count. The other 119 count cells remain blank.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1ddf418604904b84"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R15ddfa7fd3714609"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>